<commit_message>
feat: sepet hatalari ve yetkilendirme scriptleri eklendi
</commit_message>
<xml_diff>
--- a/Proje Yol Haritası ve Teknik Analiz.xlsx
+++ b/Proje Yol Haritası ve Teknik Analiz.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emiro\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emiro\Desktop\E-Commerence\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A68A7F79-6224-402E-A92C-1CA3AB8CD18E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -344,7 +344,7 @@
     <col min="4" max="4" width="27.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -355,7 +355,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -366,7 +366,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -377,7 +377,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>9</v>
       </c>

</xml_diff>